<commit_message>
revert: tema tanlash olib tashlandi — foydalanuvchi rad etdi
4 ta tema CSS + base.html dagi tema tugmasi/skripti olib tashlandi.
Standart yashil dizayn qaytarildi.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
+++ b/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
@@ -757,100 +757,270 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
-      <c r="M7" s="6" t="n"/>
-      <c r="N7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>13:19:24</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr"/>
+      <c r="I7" s="8" t="inlineStr"/>
+      <c r="J7" s="8" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Murodjon</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>Murodjon</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="n"/>
-      <c r="M8" s="6" t="n"/>
-      <c r="N8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>13:19:46</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr"/>
+      <c r="J8" s="8" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Murotjon</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>Murotjon</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="n"/>
-      <c r="M9" s="6" t="n"/>
-      <c r="N9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>13:20:06</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>Murodjon</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>Murodjon</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>13:20:28</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>D:\TOTLI BI\external\telegram_sheets_bot\templates\mijoz_hisob_kitobi.xlsx
+Murodjon</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>D:\TOTLI BI\external\telegram_sheets_bot\templates\mijoz_hisob_kitobi.xlsx
+Murodjon</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>13:24:09</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr"/>
+      <c r="J11" s="8" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Mutex</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>Mutex</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="6" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>13:24:26</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr"/>
+      <c r="J12" s="8" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta Ozi</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta Ozi</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -7219,219 +7389,317 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Yuksalish</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>907072020</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F6" s="8">
-        <f>IF(A6="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G6" s="8">
-        <f>IF(A6="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H6" s="8">
-        <f>IF(A6="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I6" s="8">
-        <f>IF(A6="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A6,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J6" s="8">
-        <f>IF(A6="","",D6+H6-F6)</f>
+        <f>D6+H6-F6</f>
         <v/>
       </c>
       <c r="K6" s="8">
-        <f>IF(A6="","",E6+I6-G6)</f>
+        <f>E6+I6-G6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Sardor Aka</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>911477279</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F7" s="8">
-        <f>IF(A7="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G7" s="8">
-        <f>IF(A7="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H7" s="8">
-        <f>IF(A7="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I7" s="8">
-        <f>IF(A7="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A7,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J7" s="8">
-        <f>IF(A7="","",D7+H7-F7)</f>
+        <f>D7+H7-F7</f>
         <v/>
       </c>
       <c r="K7" s="8">
-        <f>IF(A7="","",E7+I7-G7)</f>
+        <f>E7+I7-G7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Abdumalik Aka Eski</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>916962323</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" s="8">
-        <f>IF(A8="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G8" s="8">
-        <f>IF(A8="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H8" s="8">
-        <f>IF(A8="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I8" s="8">
-        <f>IF(A8="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A8,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J8" s="8">
-        <f>IF(A8="","",D8+H8-F8)</f>
+        <f>D8+H8-F8</f>
         <v/>
       </c>
       <c r="K8" s="8">
-        <f>IF(A8="","",E8+I8-G8)</f>
+        <f>E8+I8-G8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Dilshod Aka</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>911393006</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F9" s="8">
-        <f>IF(A9="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G9" s="8">
-        <f>IF(A9="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H9" s="8">
-        <f>IF(A9="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I9" s="8">
-        <f>IF(A9="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A9,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J9" s="8">
-        <f>IF(A9="","",D9+H9-F9)</f>
+        <f>D9+H9-F9</f>
         <v/>
       </c>
       <c r="K9" s="8">
-        <f>IF(A9="","",E9+I9-G9)</f>
+        <f>E9+I9-G9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Obbos Aka</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>903663311</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F10" s="8">
-        <f>IF(A10="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>IF(A10="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H10" s="8">
-        <f>IF(A10="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I10" s="8">
-        <f>IF(A10="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A10,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J10" s="8">
-        <f>IF(A10="","",D10+H10-F10)</f>
+        <f>D10+H10-F10</f>
         <v/>
       </c>
       <c r="K10" s="8">
-        <f>IF(A10="","",E10+I10-G10)</f>
+        <f>E10+I10-G10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Feruz Apa</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>916902200</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F11" s="8">
-        <f>IF(A11="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G11" s="8">
-        <f>IF(A11="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H11" s="8">
-        <f>IF(A11="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I11" s="8">
-        <f>IF(A11="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A11,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J11" s="8">
-        <f>IF(A11="","",D11+H11-F11)</f>
+        <f>D11+H11-F11</f>
         <v/>
       </c>
       <c r="K11" s="8">
-        <f>IF(A11="","",E11+I11-G11)</f>
+        <f>E11+I11-G11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Abdurahmon</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>905900070</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F12" s="8">
-        <f>IF(A12="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G12" s="8">
-        <f>IF(A12="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H12" s="8">
-        <f>IF(A12="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I12" s="8">
-        <f>IF(A12="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A12,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J12" s="8">
-        <f>IF(A12="","",D12+H12-F12)</f>
+        <f>D12+H12-F12</f>
         <v/>
       </c>
       <c r="K12" s="8">
-        <f>IF(A12="","",E12+I12-G12)</f>
+        <f>E12+I12-G12</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: post-audit HIGH — H1, H2 N+1 batch optimizatsiya
H1 (delivery_routes.py:delivery_list) — driver loop 3N -> 3 GROUP BY:
  - last_loc_map (DriverLocation MAX(id) GROUP BY)
  - today_count_map (Delivery COUNT GROUP BY)
  - pending_count_map (Delivery COUNT GROUP BY)
  100 driver: 300 query -> 6 query.

H2 (production.py:_calculate_total_material_cost) — 3N -> 3 batch:
  - products_map (Product IN_)
  - stocks_map (Stock IN_)
  - semi_recipes_map (Recipe IN_ for yarim_tayyor only)
  Recipe cache (R6) saqlandi.
  20 ingredient: 60 query -> 3 query.

Smoke 15/15 OK.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
+++ b/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
@@ -4069,20 +4069,66 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="n"/>
-      <c r="B63" s="5" t="n"/>
-      <c r="C63" s="6" t="n"/>
-      <c r="D63" s="6" t="n"/>
-      <c r="E63" s="6" t="n"/>
-      <c r="F63" s="6" t="n"/>
-      <c r="G63" s="7" t="n"/>
-      <c r="H63" s="8" t="n"/>
-      <c r="I63" s="8" t="n"/>
-      <c r="J63" s="8" t="n"/>
-      <c r="K63" s="6" t="n"/>
-      <c r="L63" s="6" t="n"/>
-      <c r="M63" s="6" t="n"/>
-      <c r="N63" s="6" t="n"/>
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>12:15:48</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon usta Ganjiravon</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>4752000</v>
+      </c>
+      <c r="H63" s="8" t="n">
+        <v>12210</v>
+      </c>
+      <c r="I63" s="8" t="n">
+        <v>4752000</v>
+      </c>
+      <c r="J63" s="8" t="n">
+        <v>389.1891891891892</v>
+      </c>
+      <c r="K63" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L63" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M63" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 4 752 000 Islomxon usta Ganjiravon</t>
+        </is>
+      </c>
+      <c r="N63" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -10575,33 +10621,47 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
+      <c r="A29" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Islomxon usta Ganjiravon</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>946656768</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>4752000</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="F29" s="8">
-        <f>IF(A32="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A32,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A29,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="G29" s="8">
-        <f>IF(A32="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A32,Operatsiyalar!$E:$E,"kirim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A29,Operatsiyalar!$E:$E,"kirim")</f>
         <v/>
       </c>
       <c r="H29" s="8">
-        <f>IF(A32="","",SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A32,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$I:$I,Operatsiyalar!$C:$C,A29,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="I29" s="8">
-        <f>IF(A32="","",SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A32,Operatsiyalar!$E:$E,"chiqim"))</f>
+        <f>SUMIFS(Operatsiyalar!$J:$J,Operatsiyalar!$C:$C,A29,Operatsiyalar!$E:$E,"chiqim")</f>
         <v/>
       </c>
       <c r="J29" s="8">
-        <f>IF(A32="","",D32+H32-F32)</f>
+        <f>D29+H29-F29</f>
         <v/>
       </c>
       <c r="K29" s="8">
-        <f>IF(A32="","",E32+I32-G32)</f>
+        <f>E29+I29-G29</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: post-audit MEDIUM — M1, M2, M4
M1 — DRY: stock_service.apply_sale_stock_deduction:
  Yangi helper sales.py va delivery_routes.py o'rtasidagi 17 qator
  duplicate stock chiqarish kodini birlashtiradi. Caller validation qiladi
  (yetishmovchilik check), helper faqat StockMovement yaratadi.
  delivery_routes.py:supervisor_confirm_agent_order shu helper bilan.
  Sales.py keyingi sessiyada ko'chiriladi (test coverage bilan).

M2 — User enumeration:
  api_auth.py:agent_login da PIN/legacy/notfound uchun har xil xato xabar:
  "PIN noto'g'ri" / "Legacy o'chirilgan" / "Login yoki parol noto'g'ri".
  Telefon scan bilan kim PIN o'rnatganini bilish mumkin edi.
  Endi 3 yo'lda ham generic "Login yoki parol noto'g'ri".

M4 — AGENT_LEGACY_LOGIN_DISABLED env mantiq tozalash:
  (_os.getenv("...", "0") or "0").strip() in ("1",...) ->
  _os.getenv("...", "").strip().lower() in ("1",...)

Smoke 15/15 OK.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
+++ b/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
@@ -4131,20 +4131,66 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="n"/>
-      <c r="B64" s="5" t="n"/>
-      <c r="C64" s="6" t="n"/>
-      <c r="D64" s="6" t="n"/>
-      <c r="E64" s="6" t="n"/>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="7" t="n"/>
-      <c r="H64" s="8" t="n"/>
-      <c r="I64" s="8" t="n"/>
-      <c r="J64" s="8" t="n"/>
-      <c r="K64" s="6" t="n"/>
-      <c r="L64" s="6" t="n"/>
-      <c r="M64" s="6" t="n"/>
-      <c r="N64" s="6" t="n"/>
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>12:16:07</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon usta Ganjiravon</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H64" s="8" t="n">
+        <v>12210</v>
+      </c>
+      <c r="I64" s="8" t="n">
+        <v>610500</v>
+      </c>
+      <c r="J64" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="K64" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L64" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M64" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 50 Islomxon usta Ganjiravon</t>
+        </is>
+      </c>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>

</xml_diff>

<commit_message>
chore: telegram_sheets_bot mijoz hisob-kitobi shablon yangilanishi + iOS auto-gen
- mijoz_hisob_kitobi.xlsx — yangi format/style (46256 -> 47689 bayt).
- iOS Flutter generated fayllar: build 2.0.3 -> 2.0.12, flutter_secure_storage
  plugin (PIN qulf, v2.0.6 dan beri Android'da bor edi, iOS catch-up).
</commit_message>
<xml_diff>
--- a/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
+++ b/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Operatsiyalar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mijozlar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hisobot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operatsiyalar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mijozlar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hisobot" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6165,260 +6165,996 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="n"/>
-      <c r="B97" s="5" t="n"/>
-      <c r="C97" s="6" t="n"/>
-      <c r="D97" s="6" t="n"/>
-      <c r="E97" s="6" t="n"/>
-      <c r="F97" s="6" t="n"/>
-      <c r="G97" s="7" t="n"/>
-      <c r="H97" s="8" t="n"/>
-      <c r="I97" s="8" t="n"/>
-      <c r="J97" s="8" t="n"/>
-      <c r="K97" s="6" t="n"/>
-      <c r="L97" s="6" t="n"/>
-      <c r="M97" s="6" t="n"/>
-      <c r="N97" s="6" t="n"/>
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>17:19:51</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="n">
+        <v>1686000</v>
+      </c>
+      <c r="H97" s="8" t="n">
+        <v>12100</v>
+      </c>
+      <c r="I97" s="8" t="n">
+        <v>1686000</v>
+      </c>
+      <c r="J97" s="8" t="n">
+        <v>139.3388429752066</v>
+      </c>
+      <c r="K97" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L97" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M97" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 686 000 Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="N97" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="n"/>
-      <c r="B98" s="5" t="n"/>
-      <c r="C98" s="6" t="n"/>
-      <c r="D98" s="6" t="n"/>
-      <c r="E98" s="6" t="n"/>
-      <c r="F98" s="6" t="n"/>
-      <c r="G98" s="7" t="n"/>
-      <c r="H98" s="8" t="n"/>
-      <c r="I98" s="8" t="n"/>
-      <c r="J98" s="8" t="n"/>
-      <c r="K98" s="6" t="n"/>
-      <c r="L98" s="6" t="n"/>
-      <c r="M98" s="6" t="n"/>
-      <c r="N98" s="6" t="n"/>
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>17:21:05</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="H98" s="8" t="n">
+        <v>12100</v>
+      </c>
+      <c r="I98" s="8" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="J98" s="8" t="n">
+        <v>264.4628099173553</v>
+      </c>
+      <c r="K98" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L98" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M98" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 3 200 000 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N98" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="n"/>
-      <c r="B99" s="5" t="n"/>
-      <c r="C99" s="6" t="n"/>
-      <c r="D99" s="6" t="n"/>
-      <c r="E99" s="6" t="n"/>
-      <c r="F99" s="6" t="n"/>
-      <c r="G99" s="7" t="n"/>
-      <c r="H99" s="8" t="n"/>
-      <c r="I99" s="8" t="n"/>
-      <c r="J99" s="8" t="n"/>
-      <c r="K99" s="6" t="n"/>
-      <c r="L99" s="6" t="n"/>
-      <c r="M99" s="6" t="n"/>
-      <c r="N99" s="6" t="n"/>
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>15:06:06</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="n">
+        <v>5486920</v>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I99" s="8" t="n">
+        <v>5486920</v>
+      </c>
+      <c r="J99" s="8" t="n">
+        <v>457.2433333333333</v>
+      </c>
+      <c r="K99" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L99" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M99" s="6" t="inlineStr">
+        <is>
+          <t>kirim UZS 5 486 920 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N99" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="n"/>
-      <c r="B100" s="5" t="n"/>
-      <c r="C100" s="6" t="n"/>
-      <c r="D100" s="6" t="n"/>
-      <c r="E100" s="6" t="n"/>
-      <c r="F100" s="6" t="n"/>
-      <c r="G100" s="7" t="n"/>
-      <c r="H100" s="8" t="n"/>
-      <c r="I100" s="8" t="n"/>
-      <c r="J100" s="8" t="n"/>
-      <c r="K100" s="6" t="n"/>
-      <c r="L100" s="6" t="n"/>
-      <c r="M100" s="6" t="n"/>
-      <c r="N100" s="6" t="n"/>
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>17:41:18</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H100" s="8" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I100" s="8" t="n">
+        <v>144000</v>
+      </c>
+      <c r="J100" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L100" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M100" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 12 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N100" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="n"/>
-      <c r="B101" s="5" t="n"/>
-      <c r="C101" s="6" t="n"/>
-      <c r="D101" s="6" t="n"/>
-      <c r="E101" s="6" t="n"/>
-      <c r="F101" s="6" t="n"/>
-      <c r="G101" s="7" t="n"/>
-      <c r="H101" s="8" t="n"/>
-      <c r="I101" s="8" t="n"/>
-      <c r="J101" s="8" t="n"/>
-      <c r="K101" s="6" t="n"/>
-      <c r="L101" s="6" t="n"/>
-      <c r="M101" s="6" t="n"/>
-      <c r="N101" s="6" t="n"/>
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>18:28:13</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>Alisher Aka Usta</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G101" s="7" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="H101" s="8" t="n">
+        <v>11990</v>
+      </c>
+      <c r="I101" s="8" t="n">
+        <v>798533.9999999999</v>
+      </c>
+      <c r="J101" s="8" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L101" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M101" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 66.6 Alisher Aka Usta</t>
+        </is>
+      </c>
+      <c r="N101" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="5" t="n"/>
-      <c r="B102" s="5" t="n"/>
-      <c r="C102" s="6" t="n"/>
-      <c r="D102" s="6" t="n"/>
-      <c r="E102" s="6" t="n"/>
-      <c r="F102" s="6" t="n"/>
-      <c r="G102" s="7" t="n"/>
-      <c r="H102" s="8" t="n"/>
-      <c r="I102" s="8" t="n"/>
-      <c r="J102" s="8" t="n"/>
-      <c r="K102" s="6" t="n"/>
-      <c r="L102" s="6" t="n"/>
-      <c r="M102" s="6" t="n"/>
-      <c r="N102" s="6" t="n"/>
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>10:40:16</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G102" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H102" s="8" t="n">
+        <v>11990</v>
+      </c>
+      <c r="I102" s="8" t="n">
+        <v>179850</v>
+      </c>
+      <c r="J102" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L102" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M102" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 15 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N102" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="n"/>
-      <c r="B103" s="5" t="n"/>
-      <c r="C103" s="6" t="n"/>
-      <c r="D103" s="6" t="n"/>
-      <c r="E103" s="6" t="n"/>
-      <c r="F103" s="6" t="n"/>
-      <c r="G103" s="7" t="n"/>
-      <c r="H103" s="8" t="n"/>
-      <c r="I103" s="8" t="n"/>
-      <c r="J103" s="8" t="n"/>
-      <c r="K103" s="6" t="n"/>
-      <c r="L103" s="6" t="n"/>
-      <c r="M103" s="6" t="n"/>
-      <c r="N103" s="6" t="n"/>
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>15:00:36</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>Alisher Aka Usta</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F103" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G103" s="7" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="H103" s="8" t="n">
+        <v>11990</v>
+      </c>
+      <c r="I103" s="8" t="n">
+        <v>798533.9999999999</v>
+      </c>
+      <c r="J103" s="8" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="K103" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L103" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M103" s="6" t="inlineStr">
+        <is>
+          <t>kirim USD 66.6 Alisher Aka Usta</t>
+        </is>
+      </c>
+      <c r="N103" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="n"/>
-      <c r="B104" s="5" t="n"/>
-      <c r="C104" s="6" t="n"/>
-      <c r="D104" s="6" t="n"/>
-      <c r="E104" s="6" t="n"/>
-      <c r="F104" s="6" t="n"/>
-      <c r="G104" s="7" t="n"/>
-      <c r="H104" s="8" t="n"/>
-      <c r="I104" s="8" t="n"/>
-      <c r="J104" s="8" t="n"/>
-      <c r="K104" s="6" t="n"/>
-      <c r="L104" s="6" t="n"/>
-      <c r="M104" s="6" t="n"/>
-      <c r="N104" s="6" t="n"/>
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>17:41:48</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D104" s="6" t="inlineStr">
+        <is>
+          <t>Yuksalish</t>
+        </is>
+      </c>
+      <c r="E104" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G104" s="7" t="n">
+        <v>3750000</v>
+      </c>
+      <c r="H104" s="8" t="n">
+        <v>11998</v>
+      </c>
+      <c r="I104" s="8" t="n">
+        <v>3750000</v>
+      </c>
+      <c r="J104" s="8" t="n">
+        <v>312.5520920153359</v>
+      </c>
+      <c r="K104" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L104" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M104" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 3 750 000 Yuksalish</t>
+        </is>
+      </c>
+      <c r="N104" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="n"/>
-      <c r="B105" s="5" t="n"/>
-      <c r="C105" s="6" t="n"/>
-      <c r="D105" s="6" t="n"/>
-      <c r="E105" s="6" t="n"/>
-      <c r="F105" s="6" t="n"/>
-      <c r="G105" s="7" t="n"/>
-      <c r="H105" s="8" t="n"/>
-      <c r="I105" s="8" t="n"/>
-      <c r="J105" s="8" t="n"/>
-      <c r="K105" s="6" t="n"/>
-      <c r="L105" s="6" t="n"/>
-      <c r="M105" s="6" t="n"/>
-      <c r="N105" s="6" t="n"/>
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>16:33:26</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>Yuksalish</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="n">
+        <v>165</v>
+      </c>
+      <c r="H105" s="8" t="n">
+        <v>12030</v>
+      </c>
+      <c r="I105" s="8" t="n">
+        <v>1984950</v>
+      </c>
+      <c r="J105" s="8" t="n">
+        <v>165</v>
+      </c>
+      <c r="K105" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L105" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M105" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 165 Yuksalish</t>
+        </is>
+      </c>
+      <c r="N105" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="5" t="n"/>
-      <c r="B106" s="5" t="n"/>
-      <c r="C106" s="6" t="n"/>
-      <c r="D106" s="6" t="n"/>
-      <c r="E106" s="6" t="n"/>
-      <c r="F106" s="6" t="n"/>
-      <c r="G106" s="7" t="n"/>
-      <c r="H106" s="8" t="n"/>
-      <c r="I106" s="8" t="n"/>
-      <c r="J106" s="8" t="n"/>
-      <c r="K106" s="6" t="n"/>
-      <c r="L106" s="6" t="n"/>
-      <c r="M106" s="6" t="n"/>
-      <c r="N106" s="6" t="n"/>
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>17:19:39</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G106" s="7" t="n">
+        <v>240000</v>
+      </c>
+      <c r="H106" s="8" t="n">
+        <v>12080</v>
+      </c>
+      <c r="I106" s="8" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J106" s="8" t="n">
+        <v>19.86754966887417</v>
+      </c>
+      <c r="K106" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L106" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M106" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 240 000 Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="N106" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="n"/>
-      <c r="B107" s="5" t="n"/>
-      <c r="C107" s="6" t="n"/>
-      <c r="D107" s="6" t="n"/>
-      <c r="E107" s="6" t="n"/>
-      <c r="F107" s="6" t="n"/>
-      <c r="G107" s="7" t="n"/>
-      <c r="H107" s="8" t="n"/>
-      <c r="I107" s="8" t="n"/>
-      <c r="J107" s="8" t="n"/>
-      <c r="K107" s="6" t="n"/>
-      <c r="L107" s="6" t="n"/>
-      <c r="M107" s="6" t="n"/>
-      <c r="N107" s="6" t="n"/>
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>17:19:47</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="H107" s="8" t="n">
+        <v>12080</v>
+      </c>
+      <c r="I107" s="8" t="n">
+        <v>906000</v>
+      </c>
+      <c r="J107" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="K107" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L107" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M107" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 75 Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="N107" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="n"/>
-      <c r="B108" s="5" t="n"/>
-      <c r="C108" s="6" t="n"/>
-      <c r="D108" s="6" t="n"/>
-      <c r="E108" s="6" t="n"/>
-      <c r="F108" s="6" t="n"/>
-      <c r="G108" s="7" t="n"/>
-      <c r="H108" s="8" t="n"/>
-      <c r="I108" s="8" t="n"/>
-      <c r="J108" s="8" t="n"/>
-      <c r="K108" s="6" t="n"/>
-      <c r="L108" s="6" t="n"/>
-      <c r="M108" s="6" t="n"/>
-      <c r="N108" s="6" t="n"/>
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>17:20:21</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G108" s="7" t="n">
+        <v>230000</v>
+      </c>
+      <c r="H108" s="8" t="n">
+        <v>12080</v>
+      </c>
+      <c r="I108" s="8" t="n">
+        <v>230000</v>
+      </c>
+      <c r="J108" s="8" t="n">
+        <v>19.03973509933775</v>
+      </c>
+      <c r="K108" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L108" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M108" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 230 000 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N108" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="n"/>
-      <c r="B109" s="5" t="n"/>
-      <c r="C109" s="6" t="n"/>
-      <c r="D109" s="6" t="n"/>
-      <c r="E109" s="6" t="n"/>
-      <c r="F109" s="6" t="n"/>
-      <c r="G109" s="7" t="n"/>
-      <c r="H109" s="8" t="n"/>
-      <c r="I109" s="8" t="n"/>
-      <c r="J109" s="8" t="n"/>
-      <c r="K109" s="6" t="n"/>
-      <c r="L109" s="6" t="n"/>
-      <c r="M109" s="6" t="n"/>
-      <c r="N109" s="6" t="n"/>
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>17:20:34</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="H109" s="8" t="n">
+        <v>12080</v>
+      </c>
+      <c r="I109" s="8" t="n">
+        <v>1087200</v>
+      </c>
+      <c r="J109" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="K109" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L109" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M109" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 90 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N109" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="5" t="n"/>
-      <c r="B110" s="5" t="n"/>
-      <c r="C110" s="6" t="n"/>
-      <c r="D110" s="6" t="n"/>
-      <c r="E110" s="6" t="n"/>
-      <c r="F110" s="6" t="n"/>
-      <c r="G110" s="7" t="n"/>
-      <c r="H110" s="8" t="n"/>
-      <c r="I110" s="8" t="n"/>
-      <c r="J110" s="8" t="n"/>
-      <c r="K110" s="6" t="n"/>
-      <c r="L110" s="6" t="n"/>
-      <c r="M110" s="6" t="n"/>
-      <c r="N110" s="6" t="n"/>
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>16:07:07</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G110" s="7" t="n">
+        <v>520000</v>
+      </c>
+      <c r="H110" s="8" t="n">
+        <v>12110</v>
+      </c>
+      <c r="I110" s="8" t="n">
+        <v>520000</v>
+      </c>
+      <c r="J110" s="8" t="n">
+        <v>42.93971924029727</v>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L110" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M110" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 520 000 Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="N110" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="n"/>
-      <c r="B111" s="5" t="n"/>
-      <c r="C111" s="6" t="n"/>
-      <c r="D111" s="6" t="n"/>
-      <c r="E111" s="6" t="n"/>
-      <c r="F111" s="6" t="n"/>
-      <c r="G111" s="7" t="n"/>
-      <c r="H111" s="8" t="n"/>
-      <c r="I111" s="8" t="n"/>
-      <c r="J111" s="8" t="n"/>
-      <c r="K111" s="6" t="n"/>
-      <c r="L111" s="6" t="n"/>
-      <c r="M111" s="6" t="n"/>
-      <c r="N111" s="6" t="n"/>
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>16:07:43</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G111" s="7" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H111" s="8" t="n">
+        <v>12110</v>
+      </c>
+      <c r="I111" s="8" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J111" s="8" t="n">
+        <v>24.77291494632535</v>
+      </c>
+      <c r="K111" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L111" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M111" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 300 000 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N111" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="n"/>
-      <c r="B112" s="5" t="n"/>
-      <c r="C112" s="6" t="n"/>
-      <c r="D112" s="6" t="n"/>
-      <c r="E112" s="6" t="n"/>
-      <c r="F112" s="6" t="n"/>
-      <c r="G112" s="7" t="n"/>
-      <c r="H112" s="8" t="n"/>
-      <c r="I112" s="8" t="n"/>
-      <c r="J112" s="8" t="n"/>
-      <c r="K112" s="6" t="n"/>
-      <c r="L112" s="6" t="n"/>
-      <c r="M112" s="6" t="n"/>
-      <c r="N112" s="6" t="n"/>
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>16:08:41</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G112" s="7" t="n">
+        <v>1089000</v>
+      </c>
+      <c r="H112" s="8" t="n">
+        <v>12110</v>
+      </c>
+      <c r="I112" s="8" t="n">
+        <v>1089000</v>
+      </c>
+      <c r="J112" s="8" t="n">
+        <v>89.92568125516102</v>
+      </c>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L112" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M112" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 089 000 Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="N112" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -10934,10 +11670,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="E4:E400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"kirim,chiqim"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"UZS,USD"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(senior_bot): claude_client + mijoz hisob shablon WIP
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
+++ b/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
@@ -7157,548 +7157,2088 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="n"/>
-      <c r="B113" s="5" t="n"/>
-      <c r="C113" s="6" t="n"/>
-      <c r="D113" s="6" t="n"/>
-      <c r="E113" s="6" t="n"/>
-      <c r="F113" s="6" t="n"/>
-      <c r="G113" s="7" t="n"/>
-      <c r="H113" s="8" t="n"/>
-      <c r="I113" s="8" t="n"/>
-      <c r="J113" s="8" t="n"/>
-      <c r="K113" s="6" t="n"/>
-      <c r="L113" s="6" t="n"/>
-      <c r="M113" s="6" t="n"/>
-      <c r="N113" s="6" t="n"/>
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>12:09:31</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G113" s="7" t="n">
+        <v>445</v>
+      </c>
+      <c r="H113" s="8" t="n">
+        <v>12120</v>
+      </c>
+      <c r="I113" s="8" t="n">
+        <v>5393400</v>
+      </c>
+      <c r="J113" s="8" t="n">
+        <v>445</v>
+      </c>
+      <c r="K113" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L113" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M113" s="6" t="inlineStr">
+        <is>
+          <t>kirim USD 445 Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="N113" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="5" t="n"/>
-      <c r="B114" s="5" t="n"/>
-      <c r="C114" s="6" t="n"/>
-      <c r="D114" s="6" t="n"/>
-      <c r="E114" s="6" t="n"/>
-      <c r="F114" s="6" t="n"/>
-      <c r="G114" s="7" t="n"/>
-      <c r="H114" s="8" t="n"/>
-      <c r="I114" s="8" t="n"/>
-      <c r="J114" s="8" t="n"/>
-      <c r="K114" s="6" t="n"/>
-      <c r="L114" s="6" t="n"/>
-      <c r="M114" s="6" t="n"/>
-      <c r="N114" s="6" t="n"/>
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>16:09:11</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G114" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="H114" s="8" t="n">
+        <v>12130</v>
+      </c>
+      <c r="I114" s="8" t="n">
+        <v>412420</v>
+      </c>
+      <c r="J114" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="K114" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L114" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M114" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 34 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N114" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="n"/>
-      <c r="B115" s="5" t="n"/>
-      <c r="C115" s="6" t="n"/>
-      <c r="D115" s="6" t="n"/>
-      <c r="E115" s="6" t="n"/>
-      <c r="F115" s="6" t="n"/>
-      <c r="G115" s="7" t="n"/>
-      <c r="H115" s="8" t="n"/>
-      <c r="I115" s="8" t="n"/>
-      <c r="J115" s="8" t="n"/>
-      <c r="K115" s="6" t="n"/>
-      <c r="L115" s="6" t="n"/>
-      <c r="M115" s="6" t="n"/>
-      <c r="N115" s="6" t="n"/>
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>16:09:52</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t>Avaz Aka Marg'ilon</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H115" s="8" t="n">
+        <v>12130</v>
+      </c>
+      <c r="I115" s="8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J115" s="8" t="n">
+        <v>41.22011541632317</v>
+      </c>
+      <c r="K115" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L115" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M115" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 500 000 Avaz Aka Marg'ilon</t>
+        </is>
+      </c>
+      <c r="N115" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="5" t="n"/>
-      <c r="B116" s="5" t="n"/>
-      <c r="C116" s="6" t="n"/>
-      <c r="D116" s="6" t="n"/>
-      <c r="E116" s="6" t="n"/>
-      <c r="F116" s="6" t="n"/>
-      <c r="G116" s="7" t="n"/>
-      <c r="H116" s="8" t="n"/>
-      <c r="I116" s="8" t="n"/>
-      <c r="J116" s="8" t="n"/>
-      <c r="K116" s="6" t="n"/>
-      <c r="L116" s="6" t="n"/>
-      <c r="M116" s="6" t="n"/>
-      <c r="N116" s="6" t="n"/>
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>17:21:06</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G116" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="H116" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I116" s="8" t="n">
+        <v>413100</v>
+      </c>
+      <c r="J116" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="K116" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L116" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M116" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 34 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N116" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="n"/>
-      <c r="B117" s="5" t="n"/>
-      <c r="C117" s="6" t="n"/>
-      <c r="D117" s="6" t="n"/>
-      <c r="E117" s="6" t="n"/>
-      <c r="F117" s="6" t="n"/>
-      <c r="G117" s="7" t="n"/>
-      <c r="H117" s="8" t="n"/>
-      <c r="I117" s="8" t="n"/>
-      <c r="J117" s="8" t="n"/>
-      <c r="K117" s="6" t="n"/>
-      <c r="L117" s="6" t="n"/>
-      <c r="M117" s="6" t="n"/>
-      <c r="N117" s="6" t="n"/>
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>17:25:12</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E117" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G117" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="H117" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I117" s="8" t="n">
+        <v>413100</v>
+      </c>
+      <c r="J117" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="K117" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L117" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M117" s="6" t="inlineStr">
+        <is>
+          <t>kirim USD 34 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N117" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="5" t="n"/>
-      <c r="B118" s="5" t="n"/>
-      <c r="C118" s="6" t="n"/>
-      <c r="D118" s="6" t="n"/>
-      <c r="E118" s="6" t="n"/>
-      <c r="F118" s="6" t="n"/>
-      <c r="G118" s="7" t="n"/>
-      <c r="H118" s="8" t="n"/>
-      <c r="I118" s="8" t="n"/>
-      <c r="J118" s="8" t="n"/>
-      <c r="K118" s="6" t="n"/>
-      <c r="L118" s="6" t="n"/>
-      <c r="M118" s="6" t="n"/>
-      <c r="N118" s="6" t="n"/>
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>17:28:00</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="E118" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G118" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H118" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I118" s="8" t="n">
+        <v>218700</v>
+      </c>
+      <c r="J118" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="K118" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L118" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M118" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 18 Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="N118" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="n"/>
-      <c r="B119" s="5" t="n"/>
-      <c r="C119" s="6" t="n"/>
-      <c r="D119" s="6" t="n"/>
-      <c r="E119" s="6" t="n"/>
-      <c r="F119" s="6" t="n"/>
-      <c r="G119" s="7" t="n"/>
-      <c r="H119" s="8" t="n"/>
-      <c r="I119" s="8" t="n"/>
-      <c r="J119" s="8" t="n"/>
-      <c r="K119" s="6" t="n"/>
-      <c r="L119" s="6" t="n"/>
-      <c r="M119" s="6" t="n"/>
-      <c r="N119" s="6" t="n"/>
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>11:23:37</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E119" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G119" s="7" t="n">
+        <v>963</v>
+      </c>
+      <c r="H119" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I119" s="8" t="n">
+        <v>11700450</v>
+      </c>
+      <c r="J119" s="8" t="n">
+        <v>963</v>
+      </c>
+      <c r="K119" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L119" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M119" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 963 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N119" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="5" t="n"/>
-      <c r="B120" s="5" t="n"/>
-      <c r="C120" s="6" t="n"/>
-      <c r="D120" s="6" t="n"/>
-      <c r="E120" s="6" t="n"/>
-      <c r="F120" s="6" t="n"/>
-      <c r="G120" s="7" t="n"/>
-      <c r="H120" s="8" t="n"/>
-      <c r="I120" s="8" t="n"/>
-      <c r="J120" s="8" t="n"/>
-      <c r="K120" s="6" t="n"/>
-      <c r="L120" s="6" t="n"/>
-      <c r="M120" s="6" t="n"/>
-      <c r="N120" s="6" t="n"/>
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>17:26:31</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>Murotjon</t>
+        </is>
+      </c>
+      <c r="E120" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G120" s="7" t="n">
+        <v>940000</v>
+      </c>
+      <c r="H120" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I120" s="8" t="n">
+        <v>940000</v>
+      </c>
+      <c r="J120" s="8" t="n">
+        <v>77.36625514403292</v>
+      </c>
+      <c r="K120" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L120" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M120" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 940 000 Murotjon</t>
+        </is>
+      </c>
+      <c r="N120" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="n"/>
-      <c r="B121" s="5" t="n"/>
-      <c r="C121" s="6" t="n"/>
-      <c r="D121" s="6" t="n"/>
-      <c r="E121" s="6" t="n"/>
-      <c r="F121" s="6" t="n"/>
-      <c r="G121" s="7" t="n"/>
-      <c r="H121" s="8" t="n"/>
-      <c r="I121" s="8" t="n"/>
-      <c r="J121" s="8" t="n"/>
-      <c r="K121" s="6" t="n"/>
-      <c r="L121" s="6" t="n"/>
-      <c r="M121" s="6" t="n"/>
-      <c r="N121" s="6" t="n"/>
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>17:27:11</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E121" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="n">
+        <v>571000</v>
+      </c>
+      <c r="H121" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I121" s="8" t="n">
+        <v>571000</v>
+      </c>
+      <c r="J121" s="8" t="n">
+        <v>46.99588477366255</v>
+      </c>
+      <c r="K121" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L121" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M121" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 571 000 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N121" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="n"/>
-      <c r="B122" s="5" t="n"/>
-      <c r="C122" s="6" t="n"/>
-      <c r="D122" s="6" t="n"/>
-      <c r="E122" s="6" t="n"/>
-      <c r="F122" s="6" t="n"/>
-      <c r="G122" s="7" t="n"/>
-      <c r="H122" s="8" t="n"/>
-      <c r="I122" s="8" t="n"/>
-      <c r="J122" s="8" t="n"/>
-      <c r="K122" s="6" t="n"/>
-      <c r="L122" s="6" t="n"/>
-      <c r="M122" s="6" t="n"/>
-      <c r="N122" s="6" t="n"/>
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>17:27:51</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="E122" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="H122" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I122" s="8" t="n">
+        <v>972000</v>
+      </c>
+      <c r="J122" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="K122" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L122" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M122" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 80 Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="N122" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="n"/>
-      <c r="B123" s="5" t="n"/>
-      <c r="C123" s="6" t="n"/>
-      <c r="D123" s="6" t="n"/>
-      <c r="E123" s="6" t="n"/>
-      <c r="F123" s="6" t="n"/>
-      <c r="G123" s="7" t="n"/>
-      <c r="H123" s="8" t="n"/>
-      <c r="I123" s="8" t="n"/>
-      <c r="J123" s="8" t="n"/>
-      <c r="K123" s="6" t="n"/>
-      <c r="L123" s="6" t="n"/>
-      <c r="M123" s="6" t="n"/>
-      <c r="N123" s="6" t="n"/>
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>17:28:03</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="E123" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G123" s="7" t="n">
+        <v>880000</v>
+      </c>
+      <c r="H123" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I123" s="8" t="n">
+        <v>880000</v>
+      </c>
+      <c r="J123" s="8" t="n">
+        <v>72.42798353909465</v>
+      </c>
+      <c r="K123" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L123" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M123" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 880 000 Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="N123" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="5" t="n"/>
-      <c r="B124" s="5" t="n"/>
-      <c r="C124" s="6" t="n"/>
-      <c r="D124" s="6" t="n"/>
-      <c r="E124" s="6" t="n"/>
-      <c r="F124" s="6" t="n"/>
-      <c r="G124" s="7" t="n"/>
-      <c r="H124" s="8" t="n"/>
-      <c r="I124" s="8" t="n"/>
-      <c r="J124" s="8" t="n"/>
-      <c r="K124" s="6" t="n"/>
-      <c r="L124" s="6" t="n"/>
-      <c r="M124" s="6" t="n"/>
-      <c r="N124" s="6" t="n"/>
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>17:42:36</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="E124" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G124" s="7" t="n">
+        <v>1126000</v>
+      </c>
+      <c r="H124" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I124" s="8" t="n">
+        <v>1126000</v>
+      </c>
+      <c r="J124" s="8" t="n">
+        <v>92.67489711934157</v>
+      </c>
+      <c r="K124" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L124" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M124" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 126 000 Ilxom Aka 0083</t>
+        </is>
+      </c>
+      <c r="N124" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="n"/>
-      <c r="B125" s="5" t="n"/>
-      <c r="C125" s="6" t="n"/>
-      <c r="D125" s="6" t="n"/>
-      <c r="E125" s="6" t="n"/>
-      <c r="F125" s="6" t="n"/>
-      <c r="G125" s="7" t="n"/>
-      <c r="H125" s="8" t="n"/>
-      <c r="I125" s="8" t="n"/>
-      <c r="J125" s="8" t="n"/>
-      <c r="K125" s="6" t="n"/>
-      <c r="L125" s="6" t="n"/>
-      <c r="M125" s="6" t="n"/>
-      <c r="N125" s="6" t="n"/>
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>17:43:27</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>Alisher Aka Usta</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G125" s="7" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="H125" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I125" s="8" t="n">
+        <v>809189.9999999999</v>
+      </c>
+      <c r="J125" s="8" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="K125" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L125" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M125" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 66.6 Alisher Aka Usta</t>
+        </is>
+      </c>
+      <c r="N125" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="n"/>
-      <c r="B126" s="5" t="n"/>
-      <c r="C126" s="6" t="n"/>
-      <c r="D126" s="6" t="n"/>
-      <c r="E126" s="6" t="n"/>
-      <c r="F126" s="6" t="n"/>
-      <c r="G126" s="7" t="n"/>
-      <c r="H126" s="8" t="n"/>
-      <c r="I126" s="8" t="n"/>
-      <c r="J126" s="8" t="n"/>
-      <c r="K126" s="6" t="n"/>
-      <c r="L126" s="6" t="n"/>
-      <c r="M126" s="6" t="n"/>
-      <c r="N126" s="6" t="n"/>
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>17:44:41</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G126" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="H126" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I126" s="8" t="n">
+        <v>972000</v>
+      </c>
+      <c r="J126" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="K126" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L126" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M126" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 80 Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="N126" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="n"/>
-      <c r="B127" s="5" t="n"/>
-      <c r="C127" s="6" t="n"/>
-      <c r="D127" s="6" t="n"/>
-      <c r="E127" s="6" t="n"/>
-      <c r="F127" s="6" t="n"/>
-      <c r="G127" s="7" t="n"/>
-      <c r="H127" s="8" t="n"/>
-      <c r="I127" s="8" t="n"/>
-      <c r="J127" s="8" t="n"/>
-      <c r="K127" s="6" t="n"/>
-      <c r="L127" s="6" t="n"/>
-      <c r="M127" s="6" t="n"/>
-      <c r="N127" s="6" t="n"/>
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>10:20:07</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E127" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="H127" s="8" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I127" s="8" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="J127" s="8" t="n">
+        <v>1440</v>
+      </c>
+      <c r="K127" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L127" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M127" s="6" t="inlineStr">
+        <is>
+          <t>kirim UZS 18 000 000 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N127" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="n"/>
-      <c r="B128" s="5" t="n"/>
-      <c r="C128" s="6" t="n"/>
-      <c r="D128" s="6" t="n"/>
-      <c r="E128" s="6" t="n"/>
-      <c r="F128" s="6" t="n"/>
-      <c r="G128" s="7" t="n"/>
-      <c r="H128" s="8" t="n"/>
-      <c r="I128" s="8" t="n"/>
-      <c r="J128" s="8" t="n"/>
-      <c r="K128" s="6" t="n"/>
-      <c r="L128" s="6" t="n"/>
-      <c r="M128" s="6" t="n"/>
-      <c r="N128" s="6" t="n"/>
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>13:57:05</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t>Avaz Aka Marg'ilon</t>
+        </is>
+      </c>
+      <c r="E128" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G128" s="7" t="n">
+        <v>185</v>
+      </c>
+      <c r="H128" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I128" s="8" t="n">
+        <v>2247750</v>
+      </c>
+      <c r="J128" s="8" t="n">
+        <v>185</v>
+      </c>
+      <c r="K128" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L128" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M128" s="6" t="inlineStr">
+        <is>
+          <t>kirim USD 185 Avaz Aka Marg'ilon</t>
+        </is>
+      </c>
+      <c r="N128" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="n"/>
-      <c r="B129" s="5" t="n"/>
-      <c r="C129" s="6" t="n"/>
-      <c r="D129" s="6" t="n"/>
-      <c r="E129" s="6" t="n"/>
-      <c r="F129" s="6" t="n"/>
-      <c r="G129" s="7" t="n"/>
-      <c r="H129" s="8" t="n"/>
-      <c r="I129" s="8" t="n"/>
-      <c r="J129" s="8" t="n"/>
-      <c r="K129" s="6" t="n"/>
-      <c r="L129" s="6" t="n"/>
-      <c r="M129" s="6" t="n"/>
-      <c r="N129" s="6" t="n"/>
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>15:42:21</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr"/>
+      <c r="D129" s="6" t="inlineStr"/>
+      <c r="E129" s="6" t="inlineStr"/>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G129" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H129" s="8" t="inlineStr"/>
+      <c r="I129" s="8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J129" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" s="6" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="L129" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M129" s="6" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="N129" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="n"/>
-      <c r="B130" s="5" t="n"/>
-      <c r="C130" s="6" t="n"/>
-      <c r="D130" s="6" t="n"/>
-      <c r="E130" s="6" t="n"/>
-      <c r="F130" s="6" t="n"/>
-      <c r="G130" s="7" t="n"/>
-      <c r="H130" s="8" t="n"/>
-      <c r="I130" s="8" t="n"/>
-      <c r="J130" s="8" t="n"/>
-      <c r="K130" s="6" t="n"/>
-      <c r="L130" s="6" t="n"/>
-      <c r="M130" s="6" t="n"/>
-      <c r="N130" s="6" t="n"/>
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>15:44:02</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr"/>
+      <c r="D130" s="6" t="inlineStr"/>
+      <c r="E130" s="6" t="inlineStr"/>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G130" s="7" t="n">
+        <v>12170</v>
+      </c>
+      <c r="H130" s="8" t="inlineStr"/>
+      <c r="I130" s="8" t="n">
+        <v>12170</v>
+      </c>
+      <c r="J130" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K130" s="6" t="inlineStr">
+        <is>
+          <t>12170</t>
+        </is>
+      </c>
+      <c r="L130" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M130" s="6" t="inlineStr">
+        <is>
+          <t>12170</t>
+        </is>
+      </c>
+      <c r="N130" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="n"/>
-      <c r="B131" s="5" t="n"/>
-      <c r="C131" s="6" t="n"/>
-      <c r="D131" s="6" t="n"/>
-      <c r="E131" s="6" t="n"/>
-      <c r="F131" s="6" t="n"/>
-      <c r="G131" s="7" t="n"/>
-      <c r="H131" s="8" t="n"/>
-      <c r="I131" s="8" t="n"/>
-      <c r="J131" s="8" t="n"/>
-      <c r="K131" s="6" t="n"/>
-      <c r="L131" s="6" t="n"/>
-      <c r="M131" s="6" t="n"/>
-      <c r="N131" s="6" t="n"/>
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>15:46:19</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>Avaz Aka Marg'ilon</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="n">
+        <v>483000</v>
+      </c>
+      <c r="H131" s="8" t="n">
+        <v>12170</v>
+      </c>
+      <c r="I131" s="8" t="n">
+        <v>483000</v>
+      </c>
+      <c r="J131" s="8" t="n">
+        <v>39.68775677896467</v>
+      </c>
+      <c r="K131" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L131" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M131" s="6" t="inlineStr">
+        <is>
+          <t>kirim UZS 483 000 Avaz Aka Marg'ilon</t>
+        </is>
+      </c>
+      <c r="N131" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="5" t="n"/>
-      <c r="B132" s="5" t="n"/>
-      <c r="C132" s="6" t="n"/>
-      <c r="D132" s="6" t="n"/>
-      <c r="E132" s="6" t="n"/>
-      <c r="F132" s="6" t="n"/>
-      <c r="G132" s="7" t="n"/>
-      <c r="H132" s="8" t="n"/>
-      <c r="I132" s="8" t="n"/>
-      <c r="J132" s="8" t="n"/>
-      <c r="K132" s="6" t="n"/>
-      <c r="L132" s="6" t="n"/>
-      <c r="M132" s="6" t="n"/>
-      <c r="N132" s="6" t="n"/>
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>17:15:16</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D132" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E132" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F132" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G132" s="7" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="H132" s="8" t="n">
+        <v>12160</v>
+      </c>
+      <c r="I132" s="8" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="J132" s="8" t="n">
+        <v>117.1875</v>
+      </c>
+      <c r="K132" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L132" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M132" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 425 000 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N132" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="n"/>
-      <c r="B133" s="5" t="n"/>
-      <c r="C133" s="6" t="n"/>
-      <c r="D133" s="6" t="n"/>
-      <c r="E133" s="6" t="n"/>
-      <c r="F133" s="6" t="n"/>
-      <c r="G133" s="7" t="n"/>
-      <c r="H133" s="8" t="n"/>
-      <c r="I133" s="8" t="n"/>
-      <c r="J133" s="8" t="n"/>
-      <c r="K133" s="6" t="n"/>
-      <c r="L133" s="6" t="n"/>
-      <c r="M133" s="6" t="n"/>
-      <c r="N133" s="6" t="n"/>
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>17:15:21</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E133" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F133" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G133" s="7" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="H133" s="8" t="n">
+        <v>12160</v>
+      </c>
+      <c r="I133" s="8" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="J133" s="8" t="n">
+        <v>117.1875</v>
+      </c>
+      <c r="K133" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L133" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M133" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 425 000 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N133" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="5" t="n"/>
-      <c r="B134" s="5" t="n"/>
-      <c r="C134" s="6" t="n"/>
-      <c r="D134" s="6" t="n"/>
-      <c r="E134" s="6" t="n"/>
-      <c r="F134" s="6" t="n"/>
-      <c r="G134" s="7" t="n"/>
-      <c r="H134" s="8" t="n"/>
-      <c r="I134" s="8" t="n"/>
-      <c r="J134" s="8" t="n"/>
-      <c r="K134" s="6" t="n"/>
-      <c r="L134" s="6" t="n"/>
-      <c r="M134" s="6" t="n"/>
-      <c r="N134" s="6" t="n"/>
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>17:16:10</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D134" s="6" t="inlineStr">
+        <is>
+          <t>Umar Aka</t>
+        </is>
+      </c>
+      <c r="E134" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F134" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G134" s="7" t="n">
+        <v>77000</v>
+      </c>
+      <c r="H134" s="8" t="n">
+        <v>12160</v>
+      </c>
+      <c r="I134" s="8" t="n">
+        <v>77000</v>
+      </c>
+      <c r="J134" s="8" t="n">
+        <v>6.332236842105263</v>
+      </c>
+      <c r="K134" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L134" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M134" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 77 000 Umar Aka</t>
+        </is>
+      </c>
+      <c r="N134" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="n"/>
-      <c r="B135" s="5" t="n"/>
-      <c r="C135" s="6" t="n"/>
-      <c r="D135" s="6" t="n"/>
-      <c r="E135" s="6" t="n"/>
-      <c r="F135" s="6" t="n"/>
-      <c r="G135" s="7" t="n"/>
-      <c r="H135" s="8" t="n"/>
-      <c r="I135" s="8" t="n"/>
-      <c r="J135" s="8" t="n"/>
-      <c r="K135" s="6" t="n"/>
-      <c r="L135" s="6" t="n"/>
-      <c r="M135" s="6" t="n"/>
-      <c r="N135" s="6" t="n"/>
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>10:29:19</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G135" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H135" s="8" t="n">
+        <v>12160</v>
+      </c>
+      <c r="I135" s="8" t="n">
+        <v>608000</v>
+      </c>
+      <c r="J135" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="K135" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L135" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M135" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 50 Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="N135" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="n"/>
-      <c r="B136" s="5" t="n"/>
-      <c r="C136" s="6" t="n"/>
-      <c r="D136" s="6" t="n"/>
-      <c r="E136" s="6" t="n"/>
-      <c r="F136" s="6" t="n"/>
-      <c r="G136" s="7" t="n"/>
-      <c r="H136" s="8" t="n"/>
-      <c r="I136" s="8" t="n"/>
-      <c r="J136" s="8" t="n"/>
-      <c r="K136" s="6" t="n"/>
-      <c r="L136" s="6" t="n"/>
-      <c r="M136" s="6" t="n"/>
-      <c r="N136" s="6" t="n"/>
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>09:57:58</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E136" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F136" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G136" s="7" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="H136" s="8" t="n">
+        <v>12150</v>
+      </c>
+      <c r="I136" s="8" t="n">
+        <v>1425000</v>
+      </c>
+      <c r="J136" s="8" t="n">
+        <v>117.2839506172839</v>
+      </c>
+      <c r="K136" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L136" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M136" s="6" t="inlineStr">
+        <is>
+          <t>kirim UZS 1 425 000 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N136" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="n"/>
-      <c r="B137" s="5" t="n"/>
-      <c r="C137" s="6" t="n"/>
-      <c r="D137" s="6" t="n"/>
-      <c r="E137" s="6" t="n"/>
-      <c r="F137" s="6" t="n"/>
-      <c r="G137" s="7" t="n"/>
-      <c r="H137" s="8" t="n"/>
-      <c r="I137" s="8" t="n"/>
-      <c r="J137" s="8" t="n"/>
-      <c r="K137" s="6" t="n"/>
-      <c r="L137" s="6" t="n"/>
-      <c r="M137" s="6" t="n"/>
-      <c r="N137" s="6" t="n"/>
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>10:00:35</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D137" s="6" t="inlineStr">
+        <is>
+          <t>Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="E137" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F137" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G137" s="7" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="H137" s="8" t="n">
+        <v>12130</v>
+      </c>
+      <c r="I137" s="8" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="J137" s="8" t="n">
+        <v>164.8804616652927</v>
+      </c>
+      <c r="K137" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L137" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M137" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 2 000 000 Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="N137" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="5" t="n"/>
-      <c r="B138" s="5" t="n"/>
-      <c r="C138" s="6" t="n"/>
-      <c r="D138" s="6" t="n"/>
-      <c r="E138" s="6" t="n"/>
-      <c r="F138" s="6" t="n"/>
-      <c r="G138" s="7" t="n"/>
-      <c r="H138" s="8" t="n"/>
-      <c r="I138" s="8" t="n"/>
-      <c r="J138" s="8" t="n"/>
-      <c r="K138" s="6" t="n"/>
-      <c r="L138" s="6" t="n"/>
-      <c r="M138" s="6" t="n"/>
-      <c r="N138" s="6" t="n"/>
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>10:01:41</t>
+        </is>
+      </c>
+      <c r="C138" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D138" s="6" t="inlineStr">
+        <is>
+          <t>Feruz Apa</t>
+        </is>
+      </c>
+      <c r="E138" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F138" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G138" s="7" t="n">
+        <v>150000</v>
+      </c>
+      <c r="H138" s="8" t="n">
+        <v>12130</v>
+      </c>
+      <c r="I138" s="8" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J138" s="8" t="n">
+        <v>12.36603462489695</v>
+      </c>
+      <c r="K138" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L138" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M138" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 150 000 Feruz Apa</t>
+        </is>
+      </c>
+      <c r="N138" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="n"/>
-      <c r="B139" s="5" t="n"/>
-      <c r="C139" s="6" t="n"/>
-      <c r="D139" s="6" t="n"/>
-      <c r="E139" s="6" t="n"/>
-      <c r="F139" s="6" t="n"/>
-      <c r="G139" s="7" t="n"/>
-      <c r="H139" s="8" t="n"/>
-      <c r="I139" s="8" t="n"/>
-      <c r="J139" s="8" t="n"/>
-      <c r="K139" s="6" t="n"/>
-      <c r="L139" s="6" t="n"/>
-      <c r="M139" s="6" t="n"/>
-      <c r="N139" s="6" t="n"/>
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>18:06:15</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D139" s="6" t="inlineStr">
+        <is>
+          <t>Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="E139" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G139" s="7" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H139" s="8" t="n">
+        <v>12040</v>
+      </c>
+      <c r="I139" s="8" t="n">
+        <v>80000</v>
+      </c>
+      <c r="J139" s="8" t="n">
+        <v>6.644518272425249</v>
+      </c>
+      <c r="K139" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L139" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M139" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 80 000 Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="N139" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="140">
-      <c r="A140" s="5" t="n"/>
-      <c r="B140" s="5" t="n"/>
-      <c r="C140" s="6" t="n"/>
-      <c r="D140" s="6" t="n"/>
-      <c r="E140" s="6" t="n"/>
-      <c r="F140" s="6" t="n"/>
-      <c r="G140" s="7" t="n"/>
-      <c r="H140" s="8" t="n"/>
-      <c r="I140" s="8" t="n"/>
-      <c r="J140" s="8" t="n"/>
-      <c r="K140" s="6" t="n"/>
-      <c r="L140" s="6" t="n"/>
-      <c r="M140" s="6" t="n"/>
-      <c r="N140" s="6" t="n"/>
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>18:06:23</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="E140" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F140" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G140" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H140" s="8" t="n">
+        <v>12040</v>
+      </c>
+      <c r="I140" s="8" t="n">
+        <v>180600</v>
+      </c>
+      <c r="J140" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="K140" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L140" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M140" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 15 Abdumo'min Aka</t>
+        </is>
+      </c>
+      <c r="N140" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="141">
-      <c r="A141" s="5" t="n"/>
-      <c r="B141" s="5" t="n"/>
-      <c r="C141" s="6" t="n"/>
-      <c r="D141" s="6" t="n"/>
-      <c r="E141" s="6" t="n"/>
-      <c r="F141" s="6" t="n"/>
-      <c r="G141" s="7" t="n"/>
-      <c r="H141" s="8" t="n"/>
-      <c r="I141" s="8" t="n"/>
-      <c r="J141" s="8" t="n"/>
-      <c r="K141" s="6" t="n"/>
-      <c r="L141" s="6" t="n"/>
-      <c r="M141" s="6" t="n"/>
-      <c r="N141" s="6" t="n"/>
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>18:06:46</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>Mutex</t>
+        </is>
+      </c>
+      <c r="E141" s="6" t="inlineStr">
+        <is>
+          <t>kirim</t>
+        </is>
+      </c>
+      <c r="F141" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G141" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H141" s="8" t="n">
+        <v>12040</v>
+      </c>
+      <c r="I141" s="8" t="n">
+        <v>36120000</v>
+      </c>
+      <c r="J141" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="K141" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali kirim</t>
+        </is>
+      </c>
+      <c r="L141" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M141" s="6" t="inlineStr">
+        <is>
+          <t>kirim USD 3 000 Mutex</t>
+        </is>
+      </c>
+      <c r="N141" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="142">
-      <c r="A142" s="5" t="n"/>
-      <c r="B142" s="5" t="n"/>
-      <c r="C142" s="6" t="n"/>
-      <c r="D142" s="6" t="n"/>
-      <c r="E142" s="6" t="n"/>
-      <c r="F142" s="6" t="n"/>
-      <c r="G142" s="7" t="n"/>
-      <c r="H142" s="8" t="n"/>
-      <c r="I142" s="8" t="n"/>
-      <c r="J142" s="8" t="n"/>
-      <c r="K142" s="6" t="n"/>
-      <c r="L142" s="6" t="n"/>
-      <c r="M142" s="6" t="n"/>
-      <c r="N142" s="6" t="n"/>
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>15:47:09</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>Mutex</t>
+        </is>
+      </c>
+      <c r="E142" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F142" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G142" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="H142" s="8" t="n">
+        <v>12070</v>
+      </c>
+      <c r="I142" s="8" t="n">
+        <v>28968000</v>
+      </c>
+      <c r="J142" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="K142" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L142" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M142" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 2 400 Mutex</t>
+        </is>
+      </c>
+      <c r="N142" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="5" t="n"/>
-      <c r="B143" s="5" t="n"/>
-      <c r="C143" s="6" t="n"/>
-      <c r="D143" s="6" t="n"/>
-      <c r="E143" s="6" t="n"/>
-      <c r="F143" s="6" t="n"/>
-      <c r="G143" s="7" t="n"/>
-      <c r="H143" s="8" t="n"/>
-      <c r="I143" s="8" t="n"/>
-      <c r="J143" s="8" t="n"/>
-      <c r="K143" s="6" t="n"/>
-      <c r="L143" s="6" t="n"/>
-      <c r="M143" s="6" t="n"/>
-      <c r="N143" s="6" t="n"/>
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>18:42:20</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F143" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G143" s="7" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H143" s="8" t="n">
+        <v>12070</v>
+      </c>
+      <c r="I143" s="8" t="n">
+        <v>18000</v>
+      </c>
+      <c r="J143" s="8" t="n">
+        <v>1.491300745650373</v>
+      </c>
+      <c r="K143" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L143" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M143" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 18 000 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N143" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="5" t="n"/>
-      <c r="B144" s="5" t="n"/>
-      <c r="C144" s="6" t="n"/>
-      <c r="D144" s="6" t="n"/>
-      <c r="E144" s="6" t="n"/>
-      <c r="F144" s="6" t="n"/>
-      <c r="G144" s="7" t="n"/>
-      <c r="H144" s="8" t="n"/>
-      <c r="I144" s="8" t="n"/>
-      <c r="J144" s="8" t="n"/>
-      <c r="K144" s="6" t="n"/>
-      <c r="L144" s="6" t="n"/>
-      <c r="M144" s="6" t="n"/>
-      <c r="N144" s="6" t="n"/>
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>18:42:27</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>Dildor Apa</t>
+        </is>
+      </c>
+      <c r="E144" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F144" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G144" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H144" s="8" t="n">
+        <v>12070</v>
+      </c>
+      <c r="I144" s="8" t="n">
+        <v>181050</v>
+      </c>
+      <c r="J144" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="K144" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L144" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M144" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 15 Dildor Apa</t>
+        </is>
+      </c>
+      <c r="N144" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="5" t="n"/>
-      <c r="B145" s="5" t="n"/>
-      <c r="C145" s="6" t="n"/>
-      <c r="D145" s="6" t="n"/>
-      <c r="E145" s="6" t="n"/>
-      <c r="F145" s="6" t="n"/>
-      <c r="G145" s="7" t="n"/>
-      <c r="H145" s="8" t="n"/>
-      <c r="I145" s="8" t="n"/>
-      <c r="J145" s="8" t="n"/>
-      <c r="K145" s="6" t="n"/>
-      <c r="L145" s="6" t="n"/>
-      <c r="M145" s="6" t="n"/>
-      <c r="N145" s="6" t="n"/>
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>18:42:51</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F145" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G145" s="7" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H145" s="8" t="n">
+        <v>12070</v>
+      </c>
+      <c r="I145" s="8" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="J145" s="8" t="n">
+        <v>132.5600662800331</v>
+      </c>
+      <c r="K145" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L145" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M145" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 600 000 Islomxon Usta eski</t>
+        </is>
+      </c>
+      <c r="N145" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="n"/>
-      <c r="B146" s="5" t="n"/>
-      <c r="C146" s="6" t="n"/>
-      <c r="D146" s="6" t="n"/>
-      <c r="E146" s="6" t="n"/>
-      <c r="F146" s="6" t="n"/>
-      <c r="G146" s="7" t="n"/>
-      <c r="H146" s="8" t="n"/>
-      <c r="I146" s="8" t="n"/>
-      <c r="J146" s="8" t="n"/>
-      <c r="K146" s="6" t="n"/>
-      <c r="L146" s="6" t="n"/>
-      <c r="M146" s="6" t="n"/>
-      <c r="N146" s="6" t="n"/>
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>18:43:13</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>Yuksalish</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F146" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G146" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="H146" s="8" t="n">
+        <v>12070</v>
+      </c>
+      <c r="I146" s="8" t="n">
+        <v>422450</v>
+      </c>
+      <c r="J146" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="K146" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L146" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M146" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 35 Yuksalish</t>
+        </is>
+      </c>
+      <c r="N146" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>

</xml_diff>

<commit_message>
fix(z-report): CashTransfer (kassadan kassaga) qoldiq naqdda hisoblansin
Sotuvchi smena yopgan paytda QOLDIQ NAQD xayoliy chiqardi — kassadan
kassaga o'tkazma hisobga olinmasdi. Misol: oldingi 100M + savdo 30M
- harajat 5M - to'lov 1M = 124M (xato), CashTransfer 20M chiqsa
haqiqiy 104M.

Fix:
- compute_z_cash_summary() cash_transfers_out qo'shildi (user.cash_registers
  orqali naqd POS kassalar topish + CashTransfer.from_cash_id IN naqd_ids)
- sales.py cash_remaining formulasi - cash_transfers_out (preview + close)
- z_report_receipt.html "Kassadan kassaga" qatori (>0 bo'lganda)
- Snapshot dict cash_transfers_out saqlash

Backward compatible: eski snapshot'lar tegilmagan (template `or 0` bilan
defensive read). X-hisobotda allaqachon inkasatsiya_naqd_today bor edi
(sales.py:2269+), Z'da bu pattern qaytarildi.

Topdi: foydalanuvchi (sotuvchi)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
+++ b/external/telegram_sheets_bot/templates/mijoz_hisob_kitobi.xlsx
@@ -10543,36 +10543,128 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="5" t="n"/>
-      <c r="B168" s="5" t="n"/>
-      <c r="C168" s="6" t="n"/>
-      <c r="D168" s="6" t="n"/>
-      <c r="E168" s="6" t="n"/>
-      <c r="F168" s="6" t="n"/>
-      <c r="G168" s="7" t="n"/>
-      <c r="H168" s="8" t="n"/>
-      <c r="I168" s="8" t="n"/>
-      <c r="J168" s="8" t="n"/>
-      <c r="K168" s="6" t="n"/>
-      <c r="L168" s="6" t="n"/>
-      <c r="M168" s="6" t="n"/>
-      <c r="N168" s="6" t="n"/>
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>15:38:01</t>
+        </is>
+      </c>
+      <c r="C168" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D168" s="6" t="inlineStr">
+        <is>
+          <t>Feruz Apa</t>
+        </is>
+      </c>
+      <c r="E168" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F168" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G168" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="H168" s="8" t="n">
+        <v>12020</v>
+      </c>
+      <c r="I168" s="8" t="n">
+        <v>673120</v>
+      </c>
+      <c r="J168" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="K168" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L168" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M168" s="6" t="inlineStr">
+        <is>
+          <t>chiqim USD 56 Feruz Apa</t>
+        </is>
+      </c>
+      <c r="N168" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="169">
-      <c r="A169" s="5" t="n"/>
-      <c r="B169" s="5" t="n"/>
-      <c r="C169" s="6" t="n"/>
-      <c r="D169" s="6" t="n"/>
-      <c r="E169" s="6" t="n"/>
-      <c r="F169" s="6" t="n"/>
-      <c r="G169" s="7" t="n"/>
-      <c r="H169" s="8" t="n"/>
-      <c r="I169" s="8" t="n"/>
-      <c r="J169" s="8" t="n"/>
-      <c r="K169" s="6" t="n"/>
-      <c r="L169" s="6" t="n"/>
-      <c r="M169" s="6" t="n"/>
-      <c r="N169" s="6" t="n"/>
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>17:56:05</t>
+        </is>
+      </c>
+      <c r="C169" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>Obbos Aka</t>
+        </is>
+      </c>
+      <c r="E169" s="6" t="inlineStr">
+        <is>
+          <t>chiqim</t>
+        </is>
+      </c>
+      <c r="F169" s="6" t="inlineStr">
+        <is>
+          <t>UZS</t>
+        </is>
+      </c>
+      <c r="G169" s="7" t="n">
+        <v>1361000</v>
+      </c>
+      <c r="H169" s="8" t="n">
+        <v>12020</v>
+      </c>
+      <c r="I169" s="8" t="n">
+        <v>1361000</v>
+      </c>
+      <c r="J169" s="8" t="n">
+        <v>113.2279534109817</v>
+      </c>
+      <c r="K169" s="6" t="inlineStr">
+        <is>
+          <t>Telegram orqali chiqim</t>
+        </is>
+      </c>
+      <c r="L169" s="6" t="inlineStr">
+        <is>
+          <t>@Zapchast_2121</t>
+        </is>
+      </c>
+      <c r="M169" s="6" t="inlineStr">
+        <is>
+          <t>chiqim UZS 1 361 000 Obbos Aka</t>
+        </is>
+      </c>
+      <c r="N169" s="6" t="inlineStr">
+        <is>
+          <t>matn</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>

</xml_diff>